<commit_message>
Ajustes realizados tras creación App
</commit_message>
<xml_diff>
--- a/data/planificacion.xlsx
+++ b/data/planificacion.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,6 +440,78 @@
         <is>
           <t>personas</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>46116</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>comida</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Paella de pollo</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>46116</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>cena</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Salmón a la plancha</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>comida</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Paella de pollo</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>cena</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Salmón a la plancha</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>